<commit_message>
added main modifications CHEKPOINT
</commit_message>
<xml_diff>
--- a/esempioReale.xlsx
+++ b/esempioReale.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dev/Desktop/busplan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D743B15A-3770-384E-8AE9-F4DF023001F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D6C0C7-2C63-8E45-A556-EAB1990143A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15940" xr2:uid="{738E9E6D-36A1-A142-ABA0-5C4E8C04C295}"/>
+    <workbookView xWindow="14080" yWindow="500" windowWidth="14720" windowHeight="15880" xr2:uid="{738E9E6D-36A1-A142-ABA0-5C4E8C04C295}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="49">
   <si>
     <t>IC Aldeno-Mattarello</t>
   </si>
@@ -99,9 +99,6 @@
   </si>
   <si>
     <t xml:space="preserve">IC Taio </t>
-  </si>
-  <si>
-    <t>IC Trento 7</t>
   </si>
   <si>
     <t>Nome</t>
@@ -237,7 +234,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -245,7 +242,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -589,7 +585,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D715AAA-5B5E-5C47-A463-99DCBA2CFFC9}">
-  <dimension ref="A1:D114"/>
+  <dimension ref="A1:D113"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.33203125" customWidth="1"/>
@@ -599,26 +595,26 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
         <v>44</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>45</v>
-      </c>
-      <c r="D1" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="5">
+      <c r="B2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="4">
         <v>14</v>
       </c>
     </row>
@@ -626,10 +622,10 @@
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="5">
+      <c r="B3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="4">
         <v>13</v>
       </c>
     </row>
@@ -638,9 +634,9 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="5">
+        <v>24</v>
+      </c>
+      <c r="C4" s="4">
         <v>28</v>
       </c>
     </row>
@@ -649,9 +645,9 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="5">
+        <v>25</v>
+      </c>
+      <c r="C5" s="4">
         <v>14</v>
       </c>
     </row>
@@ -660,9 +656,9 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="5">
+        <v>26</v>
+      </c>
+      <c r="C6" s="4">
         <v>13</v>
       </c>
     </row>
@@ -671,9 +667,9 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" s="5">
+        <v>27</v>
+      </c>
+      <c r="C7" s="4">
         <v>20</v>
       </c>
     </row>
@@ -682,9 +678,9 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="5">
+        <v>28</v>
+      </c>
+      <c r="C8" s="4">
         <v>14</v>
       </c>
     </row>
@@ -692,10 +688,10 @@
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="5">
+      <c r="B9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="4">
         <v>17</v>
       </c>
     </row>
@@ -704,9 +700,9 @@
         <v>8</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="5">
+        <v>30</v>
+      </c>
+      <c r="C10" s="4">
         <v>23</v>
       </c>
     </row>
@@ -714,10 +710,10 @@
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="5">
+      <c r="B11" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="4">
         <v>24</v>
       </c>
     </row>
@@ -726,9 +722,9 @@
         <v>10</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12" s="5">
+        <v>32</v>
+      </c>
+      <c r="C12" s="4">
         <v>20</v>
       </c>
     </row>
@@ -736,28 +732,28 @@
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C13" s="5">
+      <c r="B13" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="4">
         <v>22</v>
       </c>
       <c r="D13" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" s="5">
+      <c r="B14" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="4">
         <v>15</v>
       </c>
       <c r="D14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -765,9 +761,9 @@
         <v>13</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C15" s="5">
+        <v>35</v>
+      </c>
+      <c r="C15" s="4">
         <v>25</v>
       </c>
     </row>
@@ -776,9 +772,9 @@
         <v>14</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C16" s="5">
+        <v>36</v>
+      </c>
+      <c r="C16" s="4">
         <v>26</v>
       </c>
     </row>
@@ -787,9 +783,9 @@
         <v>15</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C17" s="5">
+        <v>37</v>
+      </c>
+      <c r="C17" s="4">
         <v>16</v>
       </c>
     </row>
@@ -798,9 +794,9 @@
         <v>16</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C18" s="5">
+        <v>38</v>
+      </c>
+      <c r="C18" s="4">
         <v>26</v>
       </c>
     </row>
@@ -809,9 +805,9 @@
         <v>17</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C19" s="5">
+        <v>39</v>
+      </c>
+      <c r="C19" s="4">
         <v>21</v>
       </c>
     </row>
@@ -820,9 +816,9 @@
         <v>18</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C20" s="5">
+        <v>40</v>
+      </c>
+      <c r="C20" s="4">
         <v>27</v>
       </c>
     </row>
@@ -831,9 +827,9 @@
         <v>19</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C21" s="5">
+        <v>41</v>
+      </c>
+      <c r="C21" s="4">
         <v>17</v>
       </c>
     </row>
@@ -842,301 +838,293 @@
         <v>20</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="5">
+        <v>42</v>
+      </c>
+      <c r="C22" s="4">
         <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B23" s="3"/>
-      <c r="C23" s="6">
-        <v>23</v>
-      </c>
+      <c r="A23" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="5"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C24" s="6"/>
+      <c r="C24" s="5"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C25" s="6"/>
+      <c r="C25" s="5"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C26" s="6"/>
+      <c r="C26" s="5"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C27" s="6"/>
+      <c r="C27" s="5"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C28" s="6"/>
+      <c r="C28" s="5"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C29" s="6"/>
+      <c r="C29" s="5"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C30" s="6"/>
+      <c r="C30" s="5"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C31" s="6"/>
+      <c r="C31" s="5"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C32" s="6"/>
+      <c r="C32" s="5"/>
     </row>
     <row r="33" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C33" s="6"/>
+      <c r="C33" s="5"/>
     </row>
     <row r="34" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C34" s="6"/>
+      <c r="C34" s="5"/>
     </row>
     <row r="35" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C35" s="6"/>
+      <c r="C35" s="5"/>
     </row>
     <row r="36" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C36" s="6"/>
+      <c r="C36" s="5"/>
     </row>
     <row r="37" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C37" s="6"/>
+      <c r="C37" s="5"/>
     </row>
     <row r="38" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C38" s="6"/>
+      <c r="C38" s="5"/>
     </row>
     <row r="39" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C39" s="6"/>
+      <c r="C39" s="5"/>
     </row>
     <row r="40" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C40" s="6"/>
+      <c r="C40" s="5"/>
     </row>
     <row r="41" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C41" s="6"/>
+      <c r="C41" s="5"/>
     </row>
     <row r="42" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C42" s="6"/>
+      <c r="C42" s="5"/>
     </row>
     <row r="43" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C43" s="6"/>
+      <c r="C43" s="5"/>
     </row>
     <row r="44" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C44" s="6"/>
+      <c r="C44" s="5"/>
     </row>
     <row r="45" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C45" s="6"/>
+      <c r="C45" s="5"/>
     </row>
     <row r="46" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C46" s="6"/>
+      <c r="C46" s="5"/>
     </row>
     <row r="47" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C47" s="6"/>
+      <c r="C47" s="5"/>
     </row>
     <row r="48" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C48" s="6"/>
+      <c r="C48" s="5"/>
     </row>
     <row r="49" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C49" s="6"/>
+      <c r="C49" s="5"/>
     </row>
     <row r="50" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C50" s="6"/>
+      <c r="C50" s="5"/>
     </row>
     <row r="51" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C51" s="6"/>
+      <c r="C51" s="5"/>
     </row>
     <row r="52" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C52" s="6"/>
+      <c r="C52" s="5"/>
     </row>
     <row r="53" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C53" s="6"/>
+      <c r="C53" s="5"/>
     </row>
     <row r="54" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C54" s="6"/>
+      <c r="C54" s="5"/>
     </row>
     <row r="55" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C55" s="6"/>
+      <c r="C55" s="5"/>
     </row>
     <row r="56" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C56" s="6"/>
+      <c r="C56" s="5"/>
     </row>
     <row r="57" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C57" s="6"/>
+      <c r="C57" s="5"/>
     </row>
     <row r="58" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C58" s="6"/>
+      <c r="C58" s="5"/>
     </row>
     <row r="59" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C59" s="6"/>
+      <c r="C59" s="5"/>
     </row>
     <row r="60" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C60" s="6"/>
+      <c r="C60" s="5"/>
     </row>
     <row r="61" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C61" s="6"/>
+      <c r="C61" s="5"/>
     </row>
     <row r="62" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C62" s="6"/>
+      <c r="C62" s="5"/>
     </row>
     <row r="63" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C63" s="6"/>
+      <c r="C63" s="5"/>
     </row>
     <row r="64" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C64" s="6"/>
+      <c r="C64" s="5"/>
     </row>
     <row r="65" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C65" s="6"/>
+      <c r="C65" s="5"/>
     </row>
     <row r="66" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C66" s="6"/>
+      <c r="C66" s="5"/>
     </row>
     <row r="67" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C67" s="6"/>
+      <c r="C67" s="5"/>
     </row>
     <row r="68" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C68" s="6"/>
+      <c r="C68" s="5"/>
     </row>
     <row r="69" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C69" s="6"/>
+      <c r="C69" s="5"/>
     </row>
     <row r="70" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C70" s="6"/>
+      <c r="C70" s="5"/>
     </row>
     <row r="71" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C71" s="6"/>
+      <c r="C71" s="5"/>
     </row>
     <row r="72" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C72" s="6"/>
+      <c r="C72" s="5"/>
     </row>
     <row r="73" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C73" s="6"/>
+      <c r="C73" s="5"/>
     </row>
     <row r="74" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C74" s="6"/>
+      <c r="C74" s="5"/>
     </row>
     <row r="75" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C75" s="6"/>
+      <c r="C75" s="5"/>
     </row>
     <row r="76" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C76" s="6"/>
+      <c r="C76" s="5"/>
     </row>
     <row r="77" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C77" s="6"/>
+      <c r="C77" s="5"/>
     </row>
     <row r="78" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C78" s="6"/>
+      <c r="C78" s="5"/>
     </row>
     <row r="79" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C79" s="6"/>
+      <c r="C79" s="5"/>
     </row>
     <row r="80" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C80" s="6"/>
+      <c r="C80" s="5"/>
     </row>
     <row r="81" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C81" s="6"/>
+      <c r="C81" s="5"/>
     </row>
     <row r="82" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C82" s="6"/>
+      <c r="C82" s="5"/>
     </row>
     <row r="83" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C83" s="6"/>
+      <c r="C83" s="5"/>
     </row>
     <row r="84" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C84" s="6"/>
+      <c r="C84" s="5"/>
     </row>
     <row r="85" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C85" s="6"/>
+      <c r="C85" s="5"/>
     </row>
     <row r="86" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C86" s="6"/>
+      <c r="C86" s="5"/>
     </row>
     <row r="87" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C87" s="6"/>
+      <c r="C87" s="5"/>
     </row>
     <row r="88" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C88" s="6"/>
+      <c r="C88" s="5"/>
     </row>
     <row r="89" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C89" s="6"/>
+      <c r="C89" s="5"/>
     </row>
     <row r="90" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C90" s="6"/>
+      <c r="C90" s="5"/>
     </row>
     <row r="91" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C91" s="6"/>
+      <c r="C91" s="5"/>
     </row>
     <row r="92" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C92" s="6"/>
+      <c r="C92" s="5"/>
     </row>
     <row r="93" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C93" s="6"/>
+      <c r="C93" s="5"/>
     </row>
     <row r="94" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C94" s="6"/>
+      <c r="C94" s="5"/>
     </row>
     <row r="95" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C95" s="6"/>
+      <c r="C95" s="5"/>
     </row>
     <row r="96" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C96" s="6"/>
+      <c r="C96" s="5"/>
     </row>
     <row r="97" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C97" s="6"/>
+      <c r="C97" s="5"/>
     </row>
     <row r="98" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C98" s="6"/>
+      <c r="C98" s="5"/>
     </row>
     <row r="99" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C99" s="6"/>
+      <c r="C99" s="5"/>
     </row>
     <row r="100" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C100" s="6"/>
+      <c r="C100" s="5"/>
     </row>
     <row r="101" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C101" s="6"/>
+      <c r="C101" s="5"/>
     </row>
     <row r="102" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C102" s="6"/>
+      <c r="C102" s="5"/>
     </row>
     <row r="103" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C103" s="6"/>
+      <c r="C103" s="5"/>
     </row>
     <row r="104" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C104" s="6"/>
+      <c r="C104" s="5"/>
     </row>
     <row r="105" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C105" s="6"/>
+      <c r="C105" s="5"/>
     </row>
     <row r="106" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C106" s="6"/>
+      <c r="C106" s="5"/>
     </row>
     <row r="107" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C107" s="6"/>
+      <c r="C107" s="5"/>
     </row>
     <row r="108" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C108" s="6"/>
+      <c r="C108" s="5"/>
     </row>
     <row r="109" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C109" s="6"/>
+      <c r="C109" s="5"/>
     </row>
     <row r="110" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C110" s="6"/>
+      <c r="C110" s="5"/>
     </row>
     <row r="111" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C111" s="6"/>
+      <c r="C111" s="5"/>
     </row>
     <row r="112" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C112" s="6"/>
+      <c r="C112" s="5"/>
     </row>
     <row r="113" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C113" s="6"/>
-    </row>
-    <row r="114" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C114" s="6"/>
+      <c r="C113" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>